<commit_message>
feat(rules): add R29, a wrongful charge on a purchase becomes a merchant dispute
Before, cobro indebido on a normal purchase had no rule and fell back to an
advisor. R29 opens a cobro_indebido claim for the back-office disputes queue,
never an automatic reversal or a block. The fallback is gone: every path now
ends in a rule. R29 keeps the next free id so existing ids do not move.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/matriz_decision_es.xlsx
+++ b/docs/matriz_decision_es.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayala\Projects\others\hackthon_factored_2026\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9E463D8-64FC-450C-AB83-4772F5F2C3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB43DD76-0563-4725-95B1-9CF16E8C08EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
     <sheet name="Mejoras_Slack" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Matriz!$A$4:$V$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Matriz!$A$4:$V$33</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="887" uniqueCount="495">
   <si>
     <t>Matriz de decisión: Agente de Reclamos y Disputas (Cargo no reconocido / Cobro indebido)</t>
   </si>
@@ -787,6 +787,30 @@
     <t>Par duplicado bajo y sobre el límite</t>
   </si>
   <si>
+    <t>R29</t>
+  </si>
+  <si>
+    <t>Compra reconocida con monto o cobro incorrecto (no es comisión ni duplicado)</t>
+  </si>
+  <si>
+    <t>Sí (compra)</t>
+  </si>
+  <si>
+    <t>Sí (el comercio)</t>
+  </si>
+  <si>
+    <t>Abrir reclamo por cobro indebido con evidencia precargada y derivar a back office de disputas. Sin reversión automática ni bloqueo.</t>
+  </si>
+  <si>
+    <t>Abrimos el reclamo N.º [ID] por el cobro de [comercio]. El equipo de disputas lo revisará con el comercio; plazo de respuesta [SLA].</t>
+  </si>
+  <si>
+    <t>El cliente reconoce la compra pero no el monto o el cobro (cobro mayor al acordado, suscripción cancelada, producto no recibido). Es una disputa con el comercio: el banco no revierte sin la respuesta del comercio. Numerada R29 para no cambiar los IDs existentes.</t>
+  </si>
+  <si>
+    <t>Cobro mayor al acordado; suscripción cancelada que se sigue cobrando</t>
+  </si>
+  <si>
     <t>R24</t>
   </si>
   <si>
@@ -1186,7 +1210,7 @@
     <t>Releer reclamo.estado = Open</t>
   </si>
   <si>
-    <t>R08, R18-R23</t>
+    <t>R08, R18-R23, R29</t>
   </si>
   <si>
     <t>complaints (esquema real, escritura en tabla de trabajo)</t>
@@ -1234,7 +1258,7 @@
     <t>Ficha persistida</t>
   </si>
   <si>
-    <t>R04, R06, R12, R18-R28</t>
+    <t>R04, R06, R12, R18-R29</t>
   </si>
   <si>
     <t>Salida del sistema</t>
@@ -1712,9 +1736,9 @@
     <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2021,7 +2045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V37"/>
+  <dimension ref="A1:V38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -3707,33 +3731,33 @@
         <v>240</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="22.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" ht="68.400000000000006" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>241</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>242</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>244</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>43</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>29</v>
+        <v>109</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>29</v>
+        <v>243</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>29</v>
+        <v>176</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>29</v>
+        <v>244</v>
       </c>
       <c r="J28" s="5" t="s">
         <v>29</v>
@@ -3748,115 +3772,115 @@
         <v>245</v>
       </c>
       <c r="N28" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="O28" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="P28" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="O28" s="5" t="s">
+      <c r="Q28" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="R28" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="S28" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="T28" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="U28" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="P28" s="5" t="s">
+      <c r="V28" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="Q28" s="6" t="s">
+    </row>
+    <row r="29" spans="1:22" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M29" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="N29" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="O29" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="P29" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q29" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="R28" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="S28" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="T28" s="5" t="s">
+      <c r="R29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="S29" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="T29" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="U29" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="V29" s="5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" ht="34.200000000000003" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B30" s="5" t="s">
         <v>250</v>
       </c>
-      <c r="U28" s="5" t="s">
+      <c r="C30" s="5" t="s">
         <v>251</v>
       </c>
-      <c r="V28" s="5" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="29" spans="1:22" ht="34.200000000000003" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="D29" s="5" t="str">
+      <c r="D30" s="5" t="str">
         <f>"Herramienta falla o excede tiempo; "&amp;Umbrales!$B$15&amp;" reintento con misma clave"</f>
         <v>Herramienta falla o excede tiempo; 1 reintento con misma clave</v>
       </c>
-      <c r="E29" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="K29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="L29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M29" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="N29" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="O29" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="P29" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="Q29" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="R29" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="S29" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="T29" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="U29" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="V29" s="5" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="30" spans="1:22" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>263</v>
-      </c>
       <c r="E30" s="5" t="s">
         <v>43</v>
       </c>
@@ -3882,28 +3906,28 @@
         <v>29</v>
       </c>
       <c r="M30" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="N30" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="O30" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="N30" s="5" t="s">
+      <c r="P30" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="O30" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P30" s="5" t="s">
+      <c r="Q30" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="Q30" s="7" t="s">
-        <v>43</v>
-      </c>
       <c r="R30" s="5" t="s">
-        <v>267</v>
+        <v>66</v>
       </c>
       <c r="S30" s="5" t="s">
         <v>45</v>
       </c>
       <c r="T30" s="5" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="U30" s="5" t="s">
         <v>268</v>
@@ -3917,16 +3941,16 @@
         <v>270</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>26</v>
+        <v>251</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>271</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>29</v>
@@ -3953,136 +3977,204 @@
         <v>272</v>
       </c>
       <c r="N31" s="5" t="s">
-        <v>31</v>
+        <v>273</v>
       </c>
       <c r="O31" s="5" t="s">
-        <v>273</v>
+        <v>29</v>
       </c>
       <c r="P31" s="5" t="s">
         <v>274</v>
       </c>
-      <c r="Q31" s="6" t="s">
+      <c r="Q31" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="R31" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="S31" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="T31" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="U31" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="V31" s="5" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="E32" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="R31" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="S31" s="5" t="s">
+      <c r="F32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M32" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="N32" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="O32" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="P32" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="Q32" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R32" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="S32" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="T31" s="5" t="s">
+      <c r="T32" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="U31" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="V31" s="5" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="32" spans="1:22" ht="45.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>278</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>280</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="K32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="L32" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="M32" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="N32" s="5" t="s">
+      <c r="U32" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="V32" s="5" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" ht="45.6" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M33" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="N33" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="O32" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="P32" s="5" t="s">
-        <v>283</v>
-      </c>
-      <c r="Q32" s="7" t="s">
+      <c r="O33" s="5" t="s">
+        <v>290</v>
+      </c>
+      <c r="P33" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="Q33" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="R32" s="5" t="s">
-        <v>284</v>
-      </c>
-      <c r="S32" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="T32" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="U32" s="5" t="s">
-        <v>286</v>
-      </c>
-      <c r="V32" s="5" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="21" t="s">
-        <v>289</v>
-      </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="R33" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="S33" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="T33" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="U33" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="V33" s="5" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36" s="23" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="B36" s="22"/>
       <c r="C36" s="22"/>
       <c r="D36" s="22"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="24" t="s">
-        <v>291</v>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A37" s="21" t="s">
+        <v>298</v>
       </c>
       <c r="B37" s="22"/>
       <c r="C37" s="22"/>
       <c r="D37" s="22"/>
     </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A38" s="24" t="s">
+        <v>299</v>
+      </c>
+      <c r="B38" s="22"/>
+      <c r="C38" s="22"/>
+      <c r="D38" s="22"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:V32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:V33" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="3">
-    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A38:D38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing r:id="rId1"/>
@@ -4104,252 +4196,252 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="B5" s="10">
         <v>30</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="B6" s="10">
         <v>2</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="B7" s="11">
         <v>0.7</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="B8" s="10">
         <v>2</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>317</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="B9" s="10">
         <v>120</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="B10" s="10">
         <v>1</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="34.200000000000003" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="B11" s="10">
         <v>25</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="B12" s="10">
         <v>12</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="D12" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>321</v>
-      </c>
       <c r="F12" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="B13" s="10">
         <v>10</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="B14" s="10">
         <v>3</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="B15" s="10">
         <v>1</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>
@@ -4373,58 +4465,58 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
@@ -4432,22 +4524,22 @@
         <v>118</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
@@ -4455,45 +4547,45 @@
         <v>152</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
@@ -4501,22 +4593,22 @@
         <v>98</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -4524,45 +4616,45 @@
         <v>141</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>138</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
@@ -4570,22 +4662,22 @@
         <v>63</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
@@ -4593,22 +4685,22 @@
         <v>54</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>
@@ -4628,144 +4720,144 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="B5" s="13">
         <v>686296</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="B6" s="13">
         <v>1097</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="B7" s="13">
         <v>117021</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="B8" s="13">
         <v>67095</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="B9" s="13">
         <v>24491</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="B10" s="13">
         <v>10</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="B11" s="14">
         <v>0.45</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="B12" s="13">
         <v>6</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="B13" s="15">
         <v>2E-3</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="B14" s="13">
         <v>7.2</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="B15" s="13">
         <v>4</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -4775,14 +4867,14 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="B18" s="17">
         <f>B5/B6</f>
@@ -4792,7 +4884,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="B19" s="18">
         <f>B7/B6</f>
@@ -4802,7 +4894,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="B20" s="18">
         <f>B9/B6</f>
@@ -4812,7 +4904,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="B21" s="17">
         <f>B20*B10</f>
@@ -4822,7 +4914,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="B22" s="17">
         <f>B21*B11</f>
@@ -4832,7 +4924,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="B23" s="19">
         <f>B12*B13</f>
@@ -4842,7 +4934,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="B24" s="20">
         <f>B21*B23</f>
@@ -4852,7 +4944,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="B25" s="19">
         <f>IFERROR(B24/B22,0)</f>
@@ -4862,7 +4954,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="B26" s="18">
         <f>(B22*B14+(B21-B22)*(B14-B15))/60</f>
@@ -4872,7 +4964,7 @@
     </row>
     <row r="28" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="25" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -4900,35 +4992,35 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="57" x14ac:dyDescent="0.3">
@@ -4936,22 +5028,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="79.8" x14ac:dyDescent="0.3">
@@ -4959,22 +5051,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -4982,22 +5074,22 @@
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="68.400000000000006" x14ac:dyDescent="0.3">
@@ -5005,22 +5097,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45.6" x14ac:dyDescent="0.3">
@@ -5028,22 +5120,22 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -5051,22 +5143,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -5074,22 +5166,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>470</v>
+        <v>478</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="34.200000000000003" x14ac:dyDescent="0.3">
@@ -5097,22 +5189,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
       <c r="E12" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>476</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>468</v>
-      </c>
       <c r="G12" s="5" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="45.6" x14ac:dyDescent="0.3">
@@ -5120,22 +5212,22 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="22.8" x14ac:dyDescent="0.3">
@@ -5143,22 +5235,22 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>482</v>
+        <v>490</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>485</v>
+        <v>493</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>486</v>
+        <v>494</v>
       </c>
     </row>
   </sheetData>

</xml_diff>